<commit_message>
PAUSED (task166): stage 4 round 1 reworked, every construction in the $10 million bin's middle half, waiting on a fresh reader and judge
The extension response sharpened around a refinance cover of 1.10 and the push
written half as cash-out deals, half as lower-leverage refinances: nineteen
constructions of the decisive step (bands, the data-chosen cuts 1.08 to 1.11,
the debt yield since 2023, the debt yield with the rate, the 2027 balloons
only) file 148.3 to 150.9 with their hold-out scores; the 1.25 convention, the
note-rate DSCR, the debt yield on all history, the wall's share carried to
every balloon and every balloon extended stay outside the bin. The loss is
graded to the nearest $10 million, the overlay's start is filed in the prompt,
and the extract notes file the two facts that settle Ask A's devices.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task166/golden/overlay_designation_2027.xlsx
+++ b/task166/golden/overlay_designation_2027.xlsx
@@ -26,7 +26,7 @@
     <t>Designate the overlay against fixed-rate commercial real estate</t>
   </si>
   <si>
-    <t>$1.2 billion four-year pay-fixed overlay: trade Tuesday 15 December 2026, effective Monday 4 January 2027. Positions at the close on Monday 30 November 2026.</t>
+    <t>$1.2 billion four-year pay-fixed overlay: trades Tuesday 15 December 2026, starts Monday 4 January 2027. Positions at the close on Monday 30 November 2026.</t>
   </si>
   <si>
     <t>Designated pool</t>
@@ -38,7 +38,7 @@
     <t>Averaged +200 bp loss in economic value, $ millions</t>
   </si>
   <si>
-    <t>to the nearest 25 (policy measure, section 3)</t>
+    <t>to the nearest 10 (policy measure, section 3)</t>
   </si>
   <si>
     <t>Pool</t>
@@ -65,13 +65,13 @@
     <t>Indirect auto loans</t>
   </si>
   <si>
-    <t>Losses in the table are rounded to the nearest $5 million.</t>
+    <t>Losses in the table are rounded to the nearest $10 million.</t>
   </si>
   <si>
     <t>Run-off behind each figure</t>
   </si>
   <si>
-    <t>$3.0 billion of balloons fall due from December 2026 to December 2027 (373 loans, mostly the push of December 2021 to April 2022). At the planning cycle's 6.95 per cent five-year rate about four-fifths of that principal is expected to extend 36 months at its note rate: the extension share each loan's refinance cover carries in the maturity log since 2015. Loans already extended repay at their extended maturity.</t>
+    <t>$4.7 billion of balloons fall due from December 2026 to December 2027 (659 loans, mostly the push of December 2021 to April 2022). At the planning cycle's 6.95 per cent five-year rate about three-fifths of that principal is expected to extend 36 months at its note rate: the extension share each loan's refinance cover carries in the maturity log since 2015. Loans already extended repay at their extended maturity.</t>
   </si>
   <si>
     <t>Expected to prepay about 30 per cent a year in 2027 at the planning cycle's 6.25 per cent, against about 16 per cent over the last twelve months.</t>
@@ -89,7 +89,7 @@
     <t>Hedge programme: notional in effect at each quarter-end of 2027</t>
   </si>
   <si>
-    <t>$ millions; the treasury system's ALM book with the new overlay from 4 January 2027</t>
+    <t>$ millions; the treasury system's ALM book, with the new overlay at $1.2 billion from 4 January 2027</t>
   </si>
   <si>
     <t>Part</t>
@@ -627,7 +627,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="7">
-        <v>3887.1</v>
+        <v>5292</v>
       </c>
       <c r="C8" s="8">
         <v>150</v>
@@ -658,7 +658,7 @@
         <v>1656.1</v>
       </c>
       <c r="C10" s="10">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D10">
         <v>3</v>
@@ -672,7 +672,7 @@
         <v>1660</v>
       </c>
       <c r="C11" s="10">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D11">
         <v>4</v>

</xml_diff>